<commit_message>
Add ASR with ties, AASR with ties
</commit_message>
<xml_diff>
--- a/outputs/debug/judgements/excel_overviews/gpt-4.1_vs_Llama-2-7b-chat-hf/Llama-3.1-8B-Instruct/metrics_default_vs_aae.xlsx
+++ b/outputs/debug/judgements/excel_overviews/gpt-4.1_vs_Llama-2-7b-chat-hf/Llama-3.1-8B-Instruct/metrics_default_vs_aae.xlsx
@@ -14,14 +14,20 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
   <si>
     <t>asr</t>
   </si>
   <si>
+    <t>asr_with_ties</t>
+  </si>
+  <si>
     <t>aasr</t>
   </si>
   <si>
+    <t>aasr_with_ties</t>
+  </si>
+  <si>
     <t>fr</t>
   </si>
   <si>
@@ -35,6 +41,9 @@
   </si>
   <si>
     <t>ties</t>
+  </si>
+  <si>
+    <t>smp</t>
   </si>
 </sst>
 </file>
@@ -392,10 +401,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G2"/>
+  <dimension ref="A1:J2"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:7">
+    <row r="1" spans="1:10">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -417,28 +426,46 @@
       <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
+      <c r="H1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>9</v>
+      </c>
     </row>
-    <row r="2" spans="1:7">
+    <row r="2" spans="1:10">
       <c r="A2">
         <v>0.75</v>
       </c>
       <c r="B2">
+        <v>0.7786885245901639</v>
+      </c>
+      <c r="C2">
         <v>0</v>
       </c>
-      <c r="C2">
+      <c r="D2">
+        <v>0</v>
+      </c>
+      <c r="E2">
         <v>0.7037037037037037</v>
       </c>
-      <c r="D2">
+      <c r="F2">
         <v>0.3305785123966942</v>
       </c>
-      <c r="E2">
+      <c r="G2">
         <v>108</v>
       </c>
-      <c r="F2">
+      <c r="H2">
         <v>13</v>
       </c>
-      <c r="G2">
+      <c r="I2">
         <v>14</v>
+      </c>
+      <c r="J2">
+        <v>0.8925619834710744</v>
       </c>
     </row>
   </sheetData>

</xml_diff>